<commit_message>
Nuevo form para la gestion de los archivos JSON
</commit_message>
<xml_diff>
--- a/IDIEW/bin/Debug/Plantillas/Plantilla.xlsx
+++ b/IDIEW/bin/Debug/Plantillas/Plantilla.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\capar\Documents\GitHub\IDEW\IDIEW\bin\Debug\Plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D597544D-7058-4BD4-9D8D-732879EAEE20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F962740-52DD-420B-AECB-3C03A63B5517}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{57CA8308-0047-48D7-962C-C92FD17B13F4}"/>
   </bookViews>
@@ -617,12 +617,13 @@
     <col min="8" max="8" width="15.140625" customWidth="1"/>
     <col min="9" max="9" width="19" customWidth="1"/>
     <col min="10" max="10" width="13.42578125" customWidth="1"/>
+    <col min="11" max="11" width="14.42578125" customWidth="1"/>
     <col min="13" max="13" width="14.7109375" customWidth="1"/>
     <col min="14" max="14" width="14.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:14" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" ht="23.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>

</xml_diff>